<commit_message>
fix: address reviewer comments
</commit_message>
<xml_diff>
--- a/rules/CORE-000024/negative/02/data/unit-test-coreid-CG0082-negative 2.xlsx
+++ b/rules/CORE-000024/negative/02/data/unit-test-coreid-CG0082-negative 2.xlsx
@@ -29,12 +29,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +55,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,12 +545,160 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dataset</t>
-        </is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>AEBDSYCD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AEBDSYCD</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AEBDSYCD</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
         </is>
       </c>
     </row>
@@ -868,7 +1023,7 @@
           <t>Headache</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>Nervous system disorders</t>
         </is>
@@ -943,7 +1098,7 @@
           <t>Nausea</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Gastrointestinal disorders</t>
         </is>
@@ -1018,7 +1173,7 @@
           <t>Rash</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>Skin and subcutaneous tissue disorders</t>
         </is>

</xml_diff>